<commit_message>
Update partners: add Hamblok Pissens Architecten and Bakkerij Vanderveke, add CM & Okay logos, optimize tier layout
</commit_message>
<xml_diff>
--- a/assets/partners/OVERALL RETURN PACKAGES.xlsx
+++ b/assets/partners/OVERALL RETURN PACKAGES.xlsx
@@ -1,34 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2fb8283565dcf50a/JEF/PROJECTEN/CHAUD/2026/Partners/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="227" documentId="13_ncr:1_{CC392C41-8AC3-442E-B2E3-274BFF5B5DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABE5AC1A-F9F4-49B4-856C-3386B3A17A3F}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="13_ncr:1_{CC392C41-8AC3-442E-B2E3-274BFF5B5DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB766561-2755-4698-8E5F-123373D757A7}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="4" xr2:uid="{429C2CC8-E583-4334-8721-006522640470}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="8" xr2:uid="{429C2CC8-E583-4334-8721-006522640470}"/>
   </bookViews>
   <sheets>
     <sheet name="Algemeen" sheetId="1" r:id="rId1"/>
     <sheet name="P-Productions" sheetId="9" r:id="rId2"/>
     <sheet name="MServiceS" sheetId="18" r:id="rId3"/>
-    <sheet name="EOLA Thuisverpleging" sheetId="6" r:id="rId4"/>
-    <sheet name="CDB Sports" sheetId="20" r:id="rId5"/>
-    <sheet name="KBC Vilvoorde" sheetId="7" r:id="rId6"/>
-    <sheet name="Asiat park" sheetId="17" r:id="rId7"/>
-    <sheet name="Intal Clima" sheetId="3" r:id="rId8"/>
-    <sheet name="Biowinkel" sheetId="8" r:id="rId9"/>
-    <sheet name="Rush Vilvoorde" sheetId="10" r:id="rId10"/>
-    <sheet name="Fabri Vilvoorde" sheetId="11" r:id="rId11"/>
-    <sheet name="Silke" sheetId="12" r:id="rId12"/>
-    <sheet name="Stad Vilvoorde" sheetId="19" r:id="rId13"/>
-    <sheet name="Uitleendienst Provincie" sheetId="14" r:id="rId14"/>
-    <sheet name="Drukkerij Vilvoorde" sheetId="16" r:id="rId15"/>
-    <sheet name="Cornelissen" sheetId="15" r:id="rId16"/>
+    <sheet name="Hamblok Pissens Architecten" sheetId="21" r:id="rId4"/>
+    <sheet name="EOLA Thuisverpleging" sheetId="6" r:id="rId5"/>
+    <sheet name="CDB Sports" sheetId="20" r:id="rId6"/>
+    <sheet name="KBC Vilvoorde" sheetId="7" r:id="rId7"/>
+    <sheet name="Asiat park" sheetId="17" r:id="rId8"/>
+    <sheet name="Bakkerij Vanderveke" sheetId="22" r:id="rId9"/>
+    <sheet name="Intal Clima" sheetId="3" r:id="rId10"/>
+    <sheet name="Biowinkel" sheetId="8" r:id="rId11"/>
+    <sheet name="Rush Vilvoorde" sheetId="10" r:id="rId12"/>
+    <sheet name="Fabri Vilvoorde" sheetId="11" r:id="rId13"/>
+    <sheet name="Silke" sheetId="12" r:id="rId14"/>
+    <sheet name="Stad Vilvoorde" sheetId="19" r:id="rId15"/>
+    <sheet name="Uitleendienst Provincie" sheetId="14" r:id="rId16"/>
+    <sheet name="Drukkerij Vilvoorde" sheetId="16" r:id="rId17"/>
+    <sheet name="Cornelissen" sheetId="15" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="56">
   <si>
     <t>Gouden partner</t>
   </si>
@@ -216,6 +218,12 @@
   </si>
   <si>
     <t>Drukkerij Vilvoorde (Geld)</t>
+  </si>
+  <si>
+    <t>Hamblok Pissens Architecten</t>
+  </si>
+  <si>
+    <t>Bakkerij Vanderveke</t>
   </si>
 </sst>
 </file>
@@ -227,7 +235,7 @@
     <numFmt numFmtId="164" formatCode="[$€-2]\ #,##0;[Red]\-[$€-2]\ #,##0"/>
     <numFmt numFmtId="165" formatCode="_ &quot;€&quot;\ * #,##0_ ;_ &quot;€&quot;\ * \-#,##0_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -452,7 +460,47 @@
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Valuta" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="37">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -801,6 +849,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
   <a:themeElements>
@@ -1119,15 +1171,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1B4FEA-7533-4282-B399-C4FBC0289B75}">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" customWidth="1"/>
+    <col min="4" max="4" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="6"/>
       <c r="B1" s="7" t="s">
         <v>0</v>
@@ -1139,7 +1191,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="6"/>
       <c r="B2" s="8">
         <v>5000</v>
@@ -1151,7 +1203,7 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
@@ -1159,7 +1211,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -1169,7 +1221,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>6</v>
       </c>
@@ -1177,7 +1229,7 @@
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
@@ -1189,7 +1241,7 @@
       </c>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -1203,7 +1255,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -1217,7 +1269,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
@@ -1231,7 +1283,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>11</v>
       </c>
@@ -1239,7 +1291,7 @@
       <c r="C10" s="15"/>
       <c r="D10" s="16"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
@@ -1249,7 +1301,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
@@ -1263,7 +1315,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
@@ -1273,7 +1325,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
@@ -1285,7 +1337,7 @@
       </c>
       <c r="D14" s="3"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -1293,7 +1345,7 @@
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1303,7 +1355,7 @@
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>18</v>
       </c>
@@ -1313,7 +1365,7 @@
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>19</v>
       </c>
@@ -1327,7 +1379,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>20</v>
       </c>
@@ -1341,7 +1393,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B22" s="7" t="s">
         <v>21</v>
       </c>
@@ -1352,7 +1404,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B23" s="8">
         <v>1000</v>
       </c>
@@ -1363,7 +1415,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>24</v>
       </c>
@@ -1371,7 +1423,7 @@
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>25</v>
       </c>
@@ -1385,7 +1437,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>26</v>
       </c>
@@ -1399,7 +1451,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>27</v>
       </c>
@@ -1411,7 +1463,7 @@
       </c>
       <c r="D27" s="10"/>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="13" t="s">
         <v>3</v>
       </c>
@@ -1419,7 +1471,7 @@
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>28</v>
       </c>
@@ -1433,7 +1485,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>29</v>
       </c>
@@ -1447,7 +1499,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
@@ -1461,7 +1513,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="13" t="s">
         <v>31</v>
       </c>
@@ -1469,7 +1521,7 @@
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>32</v>
       </c>
@@ -1483,7 +1535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
@@ -1495,7 +1547,7 @@
       </c>
       <c r="D34" s="10"/>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>9</v>
       </c>
@@ -1505,7 +1557,7 @@
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="14" t="s">
         <v>34</v>
       </c>
@@ -1513,7 +1565,7 @@
       <c r="C36" s="15"/>
       <c r="D36" s="16"/>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>35</v>
       </c>
@@ -1527,7 +1579,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>36</v>
       </c>
@@ -1541,7 +1593,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="15" t="s">
         <v>16</v>
       </c>
@@ -1549,7 +1601,7 @@
       <c r="C39" s="15"/>
       <c r="D39" s="16"/>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>37</v>
       </c>
@@ -1561,7 +1613,7 @@
       </c>
       <c r="D40" s="3"/>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>20</v>
       </c>
@@ -1588,12 +1640,12 @@
     <mergeCell ref="A28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:D3 C4:D4 B5:D5 D6 B10:D10 C11:D11 C13:D13 D14 B15:D15 C16:D17">
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 D6 B10:D10 C11:D11 C13:D13 D14 B15:D15 C16:D17">
-    <cfRule type="cellIs" dxfId="31" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1602,19 +1654,19 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A877D7DA-5150-4F3F-977F-3389C50F2BB8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{517E3C08-253C-4432-B829-874A8CF3AFE4}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
@@ -1626,7 +1678,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
         <v>250</v>
@@ -1634,7 +1686,7 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>24</v>
       </c>
@@ -1642,7 +1694,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -1652,7 +1704,7 @@
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -1662,7 +1714,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -1670,7 +1722,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -1680,7 +1732,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -1690,7 +1742,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -1700,7 +1752,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -1708,7 +1760,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -1718,7 +1770,7 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>34</v>
       </c>
@@ -1726,7 +1778,7 @@
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -1736,7 +1788,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
@@ -1746,7 +1798,7 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -1754,7 +1806,565 @@
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="18" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3 B6 B10">
+    <cfRule type="cellIs" dxfId="17" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD10330E-EDD8-42C0-AF81-C432A292D406}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3 B6 B10">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A877D7DA-5150-4F3F-977F-3389C50F2BB8}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3 B6 B10">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7346D4-BD50-4B91-8A74-656AB3B571D9}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -1787,20 +2397,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7346D4-BD50-4B91-8A74-656AB3B571D9}">
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBF6F122-1872-4566-B513-26C6E0599817}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
@@ -1812,15 +2422,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>24</v>
       </c>
@@ -1828,7 +2438,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -1838,7 +2448,7 @@
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -1848,7 +2458,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -1856,7 +2466,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -1866,7 +2476,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -1876,7 +2486,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -1886,7 +2496,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -1894,7 +2504,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -1904,7 +2514,7 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>34</v>
       </c>
@@ -1912,7 +2522,7 @@
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -1922,7 +2532,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
@@ -1932,7 +2542,7 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -1940,7 +2550,7 @@
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -1973,20 +2583,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBF6F122-1872-4566-B513-26C6E0599817}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46BAD7EF-AD04-4D98-9E96-01C814560907}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
@@ -1998,23 +2608,182 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
-        <v>150</v>
+        <v>1250</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="14"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="9">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A11:D11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 C4:D6 C8:D10 C12:D13">
+    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D3 B7:D7 B11:D11">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:D3 C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB21D2E-D13F-4419-BB9D-CD08BB640ED7}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="69.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -2024,7 +2793,7 @@
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -2034,7 +2803,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -2042,7 +2811,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -2052,7 +2821,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -2062,7 +2831,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -2072,7 +2841,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -2080,7 +2849,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -2090,7 +2859,7 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>34</v>
       </c>
@@ -2098,7 +2867,7 @@
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -2108,7 +2877,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
@@ -2118,7 +2887,7 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -2126,7 +2895,7 @@
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2146,12 +2915,12 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2159,20 +2928,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46BAD7EF-AD04-4D98-9E96-01C814560907}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0490E5A1-D4BE-4B8A-9186-9FCA334F545F}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="50.453125" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
+    <col min="3" max="3" width="39.453125" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
@@ -2184,182 +2953,23 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
-        <v>1250</v>
+        <v>100</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="14"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="9">
-        <v>1</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="9">
-        <v>4</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A11:D11"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D3 B7:D7 B11:D11">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:D3 B7:D7 B11:D11 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB21D2E-D13F-4419-BB9D-CD08BB640ED7}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
-  <cols>
-    <col min="1" max="1" width="69.85546875" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
-      <c r="A1" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2">
-        <v>250</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -2369,7 +2979,7 @@
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -2379,7 +2989,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -2387,7 +2997,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -2397,7 +3007,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -2407,7 +3017,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -2417,7 +3027,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -2425,7 +3035,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -2435,7 +3045,7 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>34</v>
       </c>
@@ -2443,7 +3053,7 @@
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -2453,7 +3063,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
@@ -2463,7 +3073,7 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -2471,7 +3081,7 @@
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2504,196 +3114,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0490E5A1-D4BE-4B8A-9186-9FCA334F545F}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
-  <cols>
-    <col min="1" max="1" width="50.42578125" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" customWidth="1"/>
-    <col min="3" max="3" width="39.42578125" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
-      <c r="A1" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2">
-        <v>100</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="9">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C0AA92-8BCE-4C55-ADF8-62E4EB2B05C9}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2702,15 +3126,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71D3DFA0-E12D-496E-A087-C740006ECE82}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
         <v>38</v>
       </c>
@@ -2724,7 +3148,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
         <v>5000</v>
@@ -2732,7 +3156,7 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
@@ -2740,7 +3164,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -2750,7 +3174,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>6</v>
       </c>
@@ -2758,7 +3182,7 @@
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
@@ -2768,7 +3192,7 @@
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -2778,7 +3202,7 @@
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -2788,7 +3212,7 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
@@ -2798,13 +3222,13 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="14"/>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
       <c r="D10" s="16"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
@@ -2814,7 +3238,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -2824,7 +3248,7 @@
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -2834,13 +3258,13 @@
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="15"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="16"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>17</v>
       </c>
@@ -2850,7 +3274,7 @@
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>18</v>
       </c>
@@ -2860,7 +3284,7 @@
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
@@ -2870,7 +3294,7 @@
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
@@ -2889,17 +3313,17 @@
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 C11:D13">
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3 C4:D4 B5:D5 C6:D9 B10:D10 B14:D14 C15:D18">
-    <cfRule type="cellIs" dxfId="29" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 C6:D9 B10:D10 B14:D14 C15:D18 C11:D13">
-    <cfRule type="cellIs" dxfId="28" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 C6:D9 B10:D10 C11:D13 B14:D14 C15:D18">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2910,15 +3334,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31A1B0DA-5197-4EEA-A745-F9A19DA553C9}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -2932,7 +3356,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
         <v>1250</v>
@@ -2940,7 +3364,7 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>6</v>
       </c>
@@ -2948,7 +3372,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -2958,7 +3382,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
@@ -2968,7 +3392,7 @@
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
@@ -2978,13 +3402,13 @@
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="14"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="16"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
@@ -2994,7 +3418,7 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
@@ -3004,7 +3428,7 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -3014,13 +3438,13 @@
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="15"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="16"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
@@ -3030,7 +3454,7 @@
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
@@ -3048,17 +3472,17 @@
     <mergeCell ref="A11:D11"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3 B7:D7 B11:D11">
-    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:D3 B7:D7 B11:D11 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="B3:D3 C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3067,19 +3491,19 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69D7105-E74D-4898-A220-67DDE0C4E774}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0017EAD6-EB49-454E-A1E0-468A7833EA2E}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="79.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+    <col min="3" max="3" width="30.54296875" customWidth="1"/>
+    <col min="4" max="4" width="26.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
@@ -3091,7 +3515,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
         <v>500</v>
@@ -3099,7 +3523,7 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>24</v>
       </c>
@@ -3107,7 +3531,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -3117,7 +3541,7 @@
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -3127,7 +3551,7 @@
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -3135,7 +3559,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -3145,7 +3569,7 @@
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -3155,7 +3579,7 @@
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -3165,7 +3589,7 @@
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -3173,7 +3597,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -3183,7 +3607,7 @@
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
@@ -3193,7 +3617,7 @@
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>34</v>
       </c>
@@ -3201,7 +3625,7 @@
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -3211,7 +3635,7 @@
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>36</v>
       </c>
@@ -3221,7 +3645,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>16</v>
       </c>
@@ -3229,7 +3653,7 @@
       <c r="C16" s="15"/>
       <c r="D16" s="16"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -3239,7 +3663,419 @@
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="9">
+        <v>2</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1">
+    <cfRule type="cellIs" dxfId="28" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D2">
+    <cfRule type="cellIs" dxfId="27" priority="2" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69D7105-E74D-4898-A220-67DDE0C4E774}">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2">
+        <v>500</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="9">
+        <v>2</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D2">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CB1D5B-A396-40AB-B5F4-F7FF95C5C486}">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2">
+        <v>500</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
@@ -3272,20 +4108,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CB1D5B-A396-40AB-B5F4-F7FF95C5C486}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EE9D113-A17F-4534-8B62-798E099A1B7B}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
@@ -3297,7 +4133,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
         <v>500</v>
@@ -3305,7 +4141,7 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>24</v>
       </c>
@@ -3313,7 +4149,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -3323,7 +4159,7 @@
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -3333,7 +4169,7 @@
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -3341,7 +4177,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -3351,7 +4187,7 @@
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -3361,7 +4197,7 @@
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -3371,7 +4207,7 @@
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -3379,7 +4215,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -3389,7 +4225,7 @@
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
@@ -3399,7 +4235,7 @@
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>34</v>
       </c>
@@ -3407,7 +4243,7 @@
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -3417,7 +4253,7 @@
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>36</v>
       </c>
@@ -3427,7 +4263,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>16</v>
       </c>
@@ -3435,7 +4271,7 @@
       <c r="C16" s="15"/>
       <c r="D16" s="16"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -3445,7 +4281,7 @@
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
@@ -3478,20 +4314,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EE9D113-A17F-4534-8B62-798E099A1B7B}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A66A74E2-235C-4B70-B951-F1BCEFA88BEA}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="79.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+    <col min="3" max="3" width="30.54296875" customWidth="1"/>
+    <col min="4" max="4" width="26.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
@@ -3503,7 +4339,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
         <v>500</v>
@@ -3511,7 +4347,7 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>24</v>
       </c>
@@ -3519,7 +4355,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -3529,7 +4365,7 @@
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -3539,7 +4375,7 @@
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -3547,7 +4383,7 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
@@ -3557,7 +4393,7 @@
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -3567,7 +4403,7 @@
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -3577,7 +4413,7 @@
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -3585,7 +4421,7 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
@@ -3595,7 +4431,7 @@
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
@@ -3605,7 +4441,7 @@
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>34</v>
       </c>
@@ -3613,7 +4449,7 @@
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -3623,7 +4459,7 @@
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>36</v>
       </c>
@@ -3633,7 +4469,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>16</v>
       </c>
@@ -3641,7 +4477,7 @@
       <c r="C16" s="15"/>
       <c r="D16" s="16"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -3651,7 +4487,7 @@
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
@@ -3684,23 +4520,23 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A66A74E2-235C-4B70-B951-F1BCEFA88BEA}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD27A03B-8E95-4C6C-8687-9EF4A2DDD0ED}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="79.140625" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>39</v>
@@ -3709,15 +4545,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="2">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>24</v>
       </c>
@@ -3725,27 +4561,27 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -3753,37 +4589,37 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
@@ -3791,223 +4627,17 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="9">
-        <v>2</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A13:D13"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="18" priority="1" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="17" priority="2" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{517E3C08-253C-4432-B829-874A8CF3AFE4}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
-  <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
-      <c r="A1" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2">
-        <v>250</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>5</v>
-      </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>34</v>
       </c>
@@ -4015,7 +4645,7 @@
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -4025,7 +4655,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
@@ -4035,7 +4665,7 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -4043,7 +4673,7 @@
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -4055,206 +4685,20 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="15" priority="4" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD10330E-EDD8-42C0-AF81-C432A292D406}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
-  <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
-      <c r="A1" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2">
-        <v>250</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="9">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Update lineup: add Dazzling Dimension, enlarge artist photos, and remove timetable section
</commit_message>
<xml_diff>
--- a/assets/partners/OVERALL RETURN PACKAGES.xlsx
+++ b/assets/partners/OVERALL RETURN PACKAGES.xlsx
@@ -5,32 +5,35 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2fb8283565dcf50a/JEF/PROJECTEN/CHAUD/2026/Partners/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Gedeelde drives\Jiekaa Shared\EVENT ADMINISTRATIE\CHAUD\Partners\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="13_ncr:1_{CC392C41-8AC3-442E-B2E3-274BFF5B5DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB766561-2755-4698-8E5F-123373D757A7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B431D73A-B2AC-401E-B170-CBC1CE057A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="8" xr2:uid="{429C2CC8-E583-4334-8721-006522640470}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="13" xr2:uid="{429C2CC8-E583-4334-8721-006522640470}"/>
   </bookViews>
   <sheets>
     <sheet name="Algemeen" sheetId="1" r:id="rId1"/>
     <sheet name="P-Productions" sheetId="9" r:id="rId2"/>
     <sheet name="MServiceS" sheetId="18" r:id="rId3"/>
-    <sheet name="Hamblok Pissens Architecten" sheetId="21" r:id="rId4"/>
-    <sheet name="EOLA Thuisverpleging" sheetId="6" r:id="rId5"/>
-    <sheet name="CDB Sports" sheetId="20" r:id="rId6"/>
-    <sheet name="KBC Vilvoorde" sheetId="7" r:id="rId7"/>
-    <sheet name="Asiat park" sheetId="17" r:id="rId8"/>
-    <sheet name="Bakkerij Vanderveke" sheetId="22" r:id="rId9"/>
-    <sheet name="Intal Clima" sheetId="3" r:id="rId10"/>
-    <sheet name="Biowinkel" sheetId="8" r:id="rId11"/>
-    <sheet name="Rush Vilvoorde" sheetId="10" r:id="rId12"/>
-    <sheet name="Fabri Vilvoorde" sheetId="11" r:id="rId13"/>
-    <sheet name="Silke" sheetId="12" r:id="rId14"/>
-    <sheet name="Stad Vilvoorde" sheetId="19" r:id="rId15"/>
-    <sheet name="Uitleendienst Provincie" sheetId="14" r:id="rId16"/>
-    <sheet name="Drukkerij Vilvoorde" sheetId="16" r:id="rId17"/>
-    <sheet name="Cornelissen" sheetId="15" r:id="rId18"/>
+    <sheet name="Stad Vilvoorde" sheetId="19" r:id="rId4"/>
+    <sheet name="Hamblok Pissens Architecten" sheetId="21" r:id="rId5"/>
+    <sheet name="EOLA Thuisverpleging" sheetId="6" r:id="rId6"/>
+    <sheet name="CDB Sports" sheetId="20" r:id="rId7"/>
+    <sheet name="KBC Vilvoorde" sheetId="7" r:id="rId8"/>
+    <sheet name="Asiat park" sheetId="17" r:id="rId9"/>
+    <sheet name="Bakkerij Vanderveke" sheetId="22" r:id="rId10"/>
+    <sheet name="Intal Clima" sheetId="3" r:id="rId11"/>
+    <sheet name="Biowinkel" sheetId="8" r:id="rId12"/>
+    <sheet name="Rush Vilvoorde" sheetId="10" r:id="rId13"/>
+    <sheet name="Partydeals" sheetId="26" r:id="rId14"/>
+    <sheet name="Fabri Vilvoorde" sheetId="11" r:id="rId15"/>
+    <sheet name="Silke" sheetId="12" r:id="rId16"/>
+    <sheet name="CM" sheetId="24" r:id="rId17"/>
+    <sheet name="Deans" sheetId="25" r:id="rId18"/>
+    <sheet name="Uitleendienst Provincie" sheetId="14" r:id="rId19"/>
+    <sheet name="Drukkerij Vilvoorde" sheetId="16" r:id="rId20"/>
+    <sheet name="Cornelissen" sheetId="15" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -56,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="62">
   <si>
     <t>Gouden partner</t>
   </si>
@@ -224,6 +227,24 @@
   </si>
   <si>
     <t>Bakkerij Vanderveke</t>
+  </si>
+  <si>
+    <t>CM</t>
+  </si>
+  <si>
+    <t>KBC Vilvoor</t>
+  </si>
+  <si>
+    <t>Social media, mailing</t>
+  </si>
+  <si>
+    <t>Social Media, Mailing, video</t>
+  </si>
+  <si>
+    <t>Deans</t>
+  </si>
+  <si>
+    <t>Partydeals</t>
   </si>
 </sst>
 </file>
@@ -275,7 +296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -309,6 +330,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF7F11"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -411,7 +450,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -437,6 +476,21 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -449,18 +503,302 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Valuta" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="37">
+  <dxfs count="66">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -847,10 +1185,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1204,12 +1538,12 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1222,12 +1556,12 @@
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
@@ -1284,12 +1618,12 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -1338,12 +1672,12 @@
       <c r="D14" s="3"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -1416,12 +1750,12 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
@@ -1464,12 +1798,12 @@
       <c r="D27" s="10"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
@@ -1514,12 +1848,12 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
@@ -1558,12 +1892,12 @@
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="17"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
@@ -1594,12 +1928,12 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="16"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="17"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
@@ -1640,12 +1974,12 @@
     <mergeCell ref="A28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:D3 C4:D4 B5:D5 D6 B10:D10 C11:D11 C13:D13 D14 B15:D15 C16:D17">
-    <cfRule type="cellIs" dxfId="36" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 D6 B10:D10 C11:D11 C13:D13 D14 B15:D15 C16:D17">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="64" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1654,6 +1988,192 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD27A03B-8E95-4C6C-8687-9EF4A2DDD0ED}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="19"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="15"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3 B6 B10">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{517E3C08-253C-4432-B829-874A8CF3AFE4}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1665,7 +2185,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1679,7 +2199,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -1687,12 +2207,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1702,7 +2222,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -1712,15 +2232,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -1730,7 +2250,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -1740,7 +2260,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -1750,15 +2270,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -1768,15 +2288,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -1786,7 +2306,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -1796,15 +2316,15 @@
         <v>5</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -1814,7 +2334,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1825,21 +2345,31 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="18" priority="1" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="17" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="38" priority="6" operator="greaterThan">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
+      <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD10330E-EDD8-42C0-AF81-C432A292D406}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1851,7 +2381,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1865,7 +2395,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -1873,12 +2403,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1888,7 +2418,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -1898,15 +2428,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -1916,7 +2446,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -1926,7 +2456,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -1936,15 +2466,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -1954,15 +2484,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -1972,7 +2502,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -1982,15 +2512,15 @@
         <v>5</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2000,7 +2530,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2011,21 +2541,31 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="35" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="15" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="34" priority="4" operator="greaterThan">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="33" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+      <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A877D7DA-5150-4F3F-977F-3389C50F2BB8}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2037,7 +2577,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2051,7 +2591,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2059,12 +2599,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2074,7 +2614,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -2084,15 +2624,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2102,7 +2642,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -2112,7 +2652,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -2122,15 +2662,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2140,15 +2680,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2158,7 +2698,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -2168,15 +2708,15 @@
         <v>5</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2186,7 +2726,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2197,21 +2737,208 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="30" priority="4" operator="greaterThan">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="29" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="28" priority="1" operator="equal">
+      <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A1C401E-6182-4C08-9A66-51BAD626A7CF}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="69.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="19"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="26" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7346D4-BD50-4B91-8A74-656AB3B571D9}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2223,7 +2950,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2237,7 +2964,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2245,12 +2972,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2260,7 +2987,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -2270,15 +2997,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2288,7 +3015,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -2298,7 +3025,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -2308,15 +3035,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2326,15 +3053,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2344,7 +3071,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -2354,15 +3081,15 @@
         <v>5</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2372,7 +3099,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2383,21 +3110,31 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="23" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="22" priority="4" operator="greaterThan">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="21" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+      <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBF6F122-1872-4566-B513-26C6E0599817}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2409,7 +3146,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2423,7 +3160,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>150</v>
       </c>
@@ -2431,12 +3168,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2446,7 +3183,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -2456,15 +3193,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2474,7 +3211,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -2484,7 +3221,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -2494,15 +3231,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2512,15 +3249,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2530,7 +3267,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -2540,15 +3277,15 @@
         <v>5</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2558,7 +3295,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2569,34 +3306,44 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="19" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="18" priority="4" operator="greaterThan">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+      <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46BAD7EF-AD04-4D98-9E96-01C814560907}">
-  <dimension ref="A1:D13"/>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61B18B9F-5634-4C56-8ABB-6C1C0BC7D6AD}">
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.54296875" customWidth="1"/>
-    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+    <col min="1" max="1" width="50.453125" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
+    <col min="3" max="3" width="39.453125" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
-        <v>51</v>
+      <c r="A1" s="18" t="s">
+        <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
@@ -2609,140 +3356,354 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
-        <v>1250</v>
+        <v>100</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="A3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="A6" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="14"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="9">
-        <v>1</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="A10" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="9">
-        <v>4</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="B16" s="9">
+        <v>2</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D3 B7:D7 B11:D11">
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="14" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
       <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:D3 C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="greaterThan">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A0FD04-E772-4C0C-AADA-EBFA5B4B82F1}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="69.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="19"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="15"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB21D2E-D13F-4419-BB9D-CD08BB640ED7}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2754,7 +3715,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2768,7 +3729,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2776,12 +3737,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2791,7 +3752,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -2801,15 +3762,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2819,7 +3780,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -2829,7 +3790,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -2839,15 +3800,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2857,15 +3818,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2875,7 +3836,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -2885,15 +3846,15 @@
         <v>5</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2903,7 +3864,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2914,211 +3875,26 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A12:D12"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0490E5A1-D4BE-4B8A-9186-9FCA334F545F}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="50.453125" customWidth="1"/>
-    <col min="2" max="2" width="20.453125" customWidth="1"/>
-    <col min="3" max="3" width="39.453125" customWidth="1"/>
-    <col min="4" max="4" width="29.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2">
-        <v>100</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="9">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C0AA92-8BCE-4C55-ADF8-62E4EB2B05C9}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3135,7 +3911,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3149,7 +3925,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>5000</v>
       </c>
@@ -3157,12 +3933,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3172,15 +3948,15 @@
         <v>5</v>
       </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
@@ -3190,7 +3966,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="D6" s="11"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3200,7 +3976,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="11"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -3210,7 +3986,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -3219,14 +3995,16 @@
       <c r="B9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="14"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3236,7 +4014,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="11"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -3246,7 +4024,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3256,13 +4034,13 @@
         <v>2</v>
       </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="D13" s="13"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
@@ -3272,7 +4050,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -3282,7 +4060,7 @@
         <v>5</v>
       </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+      <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -3292,7 +4070,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
+      <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
@@ -3302,7 +4080,7 @@
         <v>6</v>
       </c>
       <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
+      <c r="D18" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3313,20 +4091,225 @@
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 C11:D13">
-    <cfRule type="cellIs" dxfId="34" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3 C4:D4 B5:D5 C6:D9 B10:D10 B14:D14 C15:D18">
-    <cfRule type="cellIs" dxfId="33" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 C6:D9 B10:D10 C11:D13 B14:D14 C15:D18">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="61" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0490E5A1-D4BE-4B8A-9186-9FCA334F545F}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="50.453125" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
+    <col min="3" max="3" width="39.453125" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="19"/>
+      <c r="B2" s="2">
+        <v>100</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="14"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C0AA92-8BCE-4C55-ADF8-62E4EB2B05C9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3343,7 +4326,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3357,7 +4340,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>1250</v>
       </c>
@@ -3365,12 +4348,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3380,7 +4363,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -3390,7 +4373,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="D5" s="13"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
@@ -3399,14 +4382,16 @@
       <c r="B6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="14"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
+      <c r="A7" s="21"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="17"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -3416,7 +4401,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -3426,7 +4411,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
@@ -3436,13 +4421,13 @@
         <v>1</v>
       </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="D10" s="13"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -3452,7 +4437,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="D12" s="13"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3462,7 +4447,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="D13" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3472,17 +4457,17 @@
     <mergeCell ref="A11:D11"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3 B7:D7 B11:D11">
-    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="58" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3491,8 +4476,182 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46BAD7EF-AD04-4D98-9E96-01C814560907}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="40.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="19"/>
+      <c r="B2" s="2">
+        <v>1250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="13"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="12"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="21"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="17"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="13"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="13"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="13"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="9">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A11:D11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1">
+    <cfRule type="cellIs" dxfId="57" priority="6" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D3">
+    <cfRule type="cellIs" dxfId="56" priority="5" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:D3">
+    <cfRule type="cellIs" dxfId="55" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:D7 B11:D11">
+    <cfRule type="cellIs" dxfId="54" priority="2" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D6 C8:D10 C12:D13">
+    <cfRule type="cellIs" dxfId="52" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0017EAD6-EB49-454E-A1E0-468A7833EA2E}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="79.1796875" customWidth="1"/>
@@ -3502,7 +4661,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3516,7 +4675,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -3524,12 +4683,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3539,7 +4698,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -3549,15 +4708,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3567,7 +4726,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -3577,7 +4736,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -3587,15 +4746,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3605,90 +4764,80 @@
         <v>5</v>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="A15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
+      <c r="A16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="15"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>5</v>
+        <v>20</v>
+      </c>
+      <c r="B17" s="9">
+        <v>2</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="9">
-        <v>2</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="D17" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="28" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="27" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3696,7 +4845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69D7105-E74D-4898-A220-67DDE0C4E774}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3708,7 +4857,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3722,7 +4871,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -3730,12 +4879,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3745,7 +4894,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -3755,15 +4904,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3773,7 +4922,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -3783,7 +4932,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -3793,15 +4942,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3811,7 +4960,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -3821,15 +4970,15 @@
         <v>5</v>
       </c>
       <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -3839,7 +4988,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
@@ -3849,15 +4998,15 @@
         <v>5</v>
       </c>
       <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="D15" s="15"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -3867,7 +5016,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="D17" s="15"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
@@ -3877,7 +5026,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="D18" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3889,12 +5038,12 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3902,9 +5051,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CB1D5B-A396-40AB-B5F4-F7FF95C5C486}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
@@ -3914,7 +5063,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3928,7 +5077,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -3936,12 +5085,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3951,7 +5100,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -3961,15 +5110,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3979,7 +5128,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -3989,7 +5138,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -3999,15 +5148,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4017,90 +5166,80 @@
         <v>5</v>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="A12" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="A15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
+      <c r="A16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="15"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>5</v>
+        <v>20</v>
+      </c>
+      <c r="B17" s="9">
+        <v>2</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="9">
-        <v>2</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="D17" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4108,7 +5247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EE9D113-A17F-4534-8B62-798E099A1B7B}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4120,7 +5259,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4134,7 +5273,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -4142,12 +5281,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="A3" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4157,7 +5296,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -4167,15 +5306,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -4185,7 +5324,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -4195,7 +5334,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -4205,15 +5344,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4223,7 +5362,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -4233,15 +5372,15 @@
         <v>5</v>
       </c>
       <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -4251,7 +5390,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
@@ -4261,15 +5400,15 @@
         <v>5</v>
       </c>
       <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="D15" s="15"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -4279,7 +5418,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="D17" s="15"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
@@ -4289,7 +5428,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="D18" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4301,12 +5440,12 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="22" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="21" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4314,7 +5453,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A66A74E2-235C-4B70-B951-F1BCEFA88BEA}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4326,7 +5465,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="18" t="s">
         <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4340,7 +5479,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
+      <c r="A2" s="19"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -4348,12 +5487,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4363,7 +5502,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -4373,15 +5512,15 @@
         <v>5</v>
       </c>
       <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -4391,7 +5530,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -4401,7 +5540,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
@@ -4411,15 +5550,15 @@
         <v>5</v>
       </c>
       <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4429,7 +5568,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -4439,15 +5578,15 @@
         <v>5</v>
       </c>
       <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -4457,7 +5596,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
@@ -4467,15 +5606,15 @@
         <v>5</v>
       </c>
       <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="D15" s="15"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -4485,7 +5624,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="D17" s="15"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
@@ -4495,7 +5634,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="D18" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4507,199 +5646,13 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="2" operator="equal">
       <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD27A03B-8E95-4C6C-8687-9EF4A2DDD0ED}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="40.54296875" customWidth="1"/>
-    <col min="4" max="4" width="16.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2">
-        <v>250</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="9">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A15:D15"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: voeg partners Bakkerij Vanderveken, Duvel Moortgat en Lammekeshoeve toe
</commit_message>
<xml_diff>
--- a/assets/partners/OVERALL RETURN PACKAGES.xlsx
+++ b/assets/partners/OVERALL RETURN PACKAGES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Gedeelde drives\Jiekaa Shared\EVENT ADMINISTRATIE\CHAUD\Partners\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B431D73A-B2AC-401E-B170-CBC1CE057A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0D6810-E73D-4A82-A9C2-FE23ECDC631B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="13" xr2:uid="{429C2CC8-E583-4334-8721-006522640470}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="15" activeTab="19" xr2:uid="{429C2CC8-E583-4334-8721-006522640470}"/>
   </bookViews>
   <sheets>
     <sheet name="Algemeen" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,12 @@
     <sheet name="Silke" sheetId="12" r:id="rId16"/>
     <sheet name="CM" sheetId="24" r:id="rId17"/>
     <sheet name="Deans" sheetId="25" r:id="rId18"/>
-    <sheet name="Uitleendienst Provincie" sheetId="14" r:id="rId19"/>
-    <sheet name="Drukkerij Vilvoorde" sheetId="16" r:id="rId20"/>
-    <sheet name="Cornelissen" sheetId="15" r:id="rId21"/>
+    <sheet name="Vanderveke" sheetId="27" r:id="rId19"/>
+    <sheet name="Lammekeshoeve" sheetId="29" r:id="rId20"/>
+    <sheet name="Duvel Moortgat" sheetId="28" r:id="rId21"/>
+    <sheet name="Uitleendienst Provincie" sheetId="14" r:id="rId22"/>
+    <sheet name="Drukkerij Vilvoorde" sheetId="16" r:id="rId23"/>
+    <sheet name="Cornelissen" sheetId="15" r:id="rId24"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -59,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="64">
   <si>
     <t>Gouden partner</t>
   </si>
@@ -245,6 +248,12 @@
   </si>
   <si>
     <t>Partydeals</t>
+  </si>
+  <si>
+    <t>Duvel Moortgat</t>
+  </si>
+  <si>
+    <t>Lammekeshoeve</t>
   </si>
 </sst>
 </file>
@@ -485,12 +494,6 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -503,12 +506,138 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Valuta" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="66">
+  <dxfs count="78">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1538,12 +1667,12 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1556,12 +1685,12 @@
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
@@ -1618,12 +1747,12 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -1672,12 +1801,12 @@
       <c r="D14" s="3"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -1750,12 +1879,12 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
@@ -1798,12 +1927,12 @@
       <c r="D27" s="10"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
@@ -1848,12 +1977,12 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="20" t="s">
+      <c r="A32" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
@@ -1892,12 +2021,12 @@
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="17"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="21"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
@@ -1928,12 +2057,12 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="17"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="21"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
@@ -1974,12 +2103,12 @@
     <mergeCell ref="A28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:D3 C4:D4 B5:D5 D6 B10:D10 C11:D11 C13:D13 D14 B15:D15 C16:D17">
-    <cfRule type="cellIs" dxfId="65" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 D6 B10:D10 C11:D11 C13:D13 D14 B15:D15 C16:D17">
-    <cfRule type="cellIs" dxfId="64" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="76" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1999,7 +2128,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2013,7 +2142,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2021,12 +2150,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2049,12 +2178,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2087,12 +2216,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2105,12 +2234,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2133,12 +2262,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2160,12 +2289,12 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3 C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3 B6 B10">
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2185,7 +2314,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2199,7 +2328,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2207,12 +2336,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2235,12 +2364,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2273,12 +2402,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2291,12 +2420,12 @@
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2319,12 +2448,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2346,22 +2475,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="38" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="50" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2381,7 +2510,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2395,7 +2524,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2403,12 +2532,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2431,12 +2560,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2469,12 +2598,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2487,12 +2616,12 @@
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2515,12 +2644,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2542,22 +2671,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="35" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="34" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="46" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="33" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2577,7 +2706,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2591,7 +2720,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2599,12 +2728,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2627,12 +2756,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2665,12 +2794,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2683,12 +2812,12 @@
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2711,12 +2840,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -2738,22 +2867,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="30" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="29" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="28" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2773,7 +2902,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2787,7 +2916,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2795,12 +2924,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -2823,12 +2952,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2861,12 +2990,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -2879,12 +3008,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -2915,22 +3044,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="26" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2950,7 +3079,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2964,7 +3093,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -2972,12 +3101,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3000,12 +3129,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3038,12 +3167,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3056,12 +3185,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3084,12 +3213,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -3111,22 +3240,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="23" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="22" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="34" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="21" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3146,7 +3275,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3160,7 +3289,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>150</v>
       </c>
@@ -3168,12 +3297,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3196,12 +3325,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3234,12 +3363,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3252,12 +3381,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3280,12 +3409,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -3307,22 +3436,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="19" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="18" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3342,7 +3471,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3356,7 +3485,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>100</v>
       </c>
@@ -3364,12 +3493,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3392,12 +3521,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3430,12 +3559,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3448,12 +3577,12 @@
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3476,12 +3605,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -3503,22 +3632,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="14" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3538,7 +3667,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3552,7 +3681,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -3560,12 +3689,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3588,12 +3717,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3626,12 +3755,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3644,12 +3773,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3680,22 +3809,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="22" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3704,7 +3833,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB21D2E-D13F-4419-BB9D-CD08BB640ED7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA6241D-C9F3-498B-894F-5D087B0E7C5B}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3715,8 +3844,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
-        <v>52</v>
+      <c r="A1" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
@@ -3729,7 +3858,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>250</v>
       </c>
@@ -3737,12 +3866,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3765,12 +3894,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -3803,12 +3932,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -3818,15 +3947,15 @@
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="14"/>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -3849,12 +3978,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -3876,22 +4005,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3911,7 +4040,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3925,7 +4054,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>5000</v>
       </c>
@@ -3933,12 +4062,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -3951,12 +4080,12 @@
       <c r="D4" s="11"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
@@ -4001,10 +4130,10 @@
       <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="21"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="A10" s="19"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4037,10 +4166,10 @@
       <c r="D13" s="13"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="16"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
@@ -4091,17 +4220,17 @@
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 C11:D13">
-    <cfRule type="cellIs" dxfId="63" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3 C4:D4 B5:D5 C6:D9 B10:D10 B14:D14 C15:D18">
-    <cfRule type="cellIs" dxfId="62" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D4 B5:D5 C6:D9 B10:D10 C11:D13 B14:D14 C15:D18">
-    <cfRule type="cellIs" dxfId="61" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="73" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4110,6 +4239,594 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAFA9CFF-7A8B-4229-BF04-2FA5E966D278}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="69.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="17"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A15:D15"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DCC9EB-E1BF-4AFF-8F8E-F706975E9046}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="69.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="17"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="14" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB21D2E-D13F-4419-BB9D-CD08BB640ED7}">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="69.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A1" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="17"/>
+      <c r="B2" s="2">
+        <v>250</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="14"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1 B1:D3">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6 B10">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0490E5A1-D4BE-4B8A-9186-9FCA334F545F}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4121,7 +4838,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4135,7 +4852,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>100</v>
       </c>
@@ -4143,12 +4860,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4171,12 +4888,12 @@
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -4209,12 +4926,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4227,12 +4944,12 @@
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -4255,12 +4972,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -4282,22 +4999,22 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 B1:D3">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 B10">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D5 B6:D6 C7:D9 B10:D10 C11:D11">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4305,7 +5022,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C0AA92-8BCE-4C55-ADF8-62E4EB2B05C9}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4326,7 +5043,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4340,7 +5057,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>1250</v>
       </c>
@@ -4348,12 +5065,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4388,10 +5105,10 @@
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="21"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="17"/>
+      <c r="A7" s="19"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="21"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -4424,10 +5141,10 @@
       <c r="D10" s="13"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="21"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -4457,17 +5174,17 @@
     <mergeCell ref="A11:D11"/>
   </mergeCells>
   <conditionalFormatting sqref="A1 C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3 B7:D7 B11:D11">
-    <cfRule type="cellIs" dxfId="59" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3 C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
-    <cfRule type="cellIs" dxfId="58" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="70" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4487,7 +5204,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4501,7 +5218,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>1250</v>
       </c>
@@ -4509,12 +5226,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4547,10 +5264,10 @@
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="21"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="17"/>
+      <c r="A7" s="19"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="21"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -4583,10 +5300,10 @@
       <c r="D10" s="13"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="21"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
@@ -4616,32 +5333,32 @@
     <mergeCell ref="A11:D11"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="57" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="6" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D3">
-    <cfRule type="cellIs" dxfId="56" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="5" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D3">
-    <cfRule type="cellIs" dxfId="55" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="67" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7 B11:D11">
-    <cfRule type="cellIs" dxfId="54" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D6 B7:D7 C8:D10 B11:D11 C12:D13">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="65" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:D6 C8:D10 C12:D13">
-    <cfRule type="cellIs" dxfId="52" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="3" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4661,7 +5378,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4675,7 +5392,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -4683,12 +5400,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4711,12 +5428,12 @@
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -4749,12 +5466,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4767,12 +5484,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -4795,12 +5512,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -4832,12 +5549,12 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="51" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4857,7 +5574,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4871,7 +5588,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -4879,12 +5596,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -4907,12 +5624,12 @@
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -4945,12 +5662,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -4973,12 +5690,12 @@
       <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="17"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="21"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -5001,12 +5718,12 @@
       <c r="D15" s="15"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -5038,12 +5755,12 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5063,7 +5780,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -5077,7 +5794,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -5085,12 +5802,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -5113,12 +5830,12 @@
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -5151,12 +5868,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -5169,12 +5886,12 @@
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
@@ -5197,12 +5914,12 @@
       <c r="D14" s="15"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
@@ -5234,12 +5951,12 @@
     <mergeCell ref="A12:D12"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5259,7 +5976,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -5273,7 +5990,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -5281,12 +5998,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -5309,12 +6026,12 @@
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -5347,12 +6064,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -5375,12 +6092,12 @@
       <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="17"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="21"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -5403,12 +6120,12 @@
       <c r="D15" s="15"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -5440,12 +6157,12 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="45" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="44" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5465,7 +6182,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -5479,7 +6196,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
+      <c r="A2" s="17"/>
       <c r="B2" s="2">
         <v>500</v>
       </c>
@@ -5487,12 +6204,12 @@
       <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -5515,12 +6232,12 @@
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -5553,12 +6270,12 @@
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -5581,12 +6298,12 @@
       <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="17"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="21"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -5609,12 +6326,12 @@
       <c r="D15" s="15"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
@@ -5646,12 +6363,12 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="1" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:D2">
-    <cfRule type="cellIs" dxfId="42" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>